<commit_message>
nearly done for jonas final
</commit_message>
<xml_diff>
--- a/data/5_results/no_prompt/result_llama_no_prompt_5.xlsx
+++ b/data/5_results/no_prompt/result_llama_no_prompt_5.xlsx
@@ -427,19 +427,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="5" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,17 +502,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0,934</t>
+          <t>0,913</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0,951</t>
+          <t>0,942</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,942</t>
+          <t>0,927</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2668,000</t>
+          <t>414,000</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -531,13 +531,13 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2536</v>
+        <v>390</v>
       </c>
       <c r="I2" t="n">
-        <v>179</v>
+        <v>37</v>
       </c>
       <c r="J2" t="n">
-        <v>132</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -548,42 +548,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0,936</t>
+          <t>0,905</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0,945</t>
+          <t>0,911</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0,940</t>
+          <t>0,908</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0,998</t>
+          <t>0,999</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2624,000</t>
+          <t>416,000</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0,56</t>
+          <t>0,58</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2480</v>
+        <v>379</v>
       </c>
       <c r="I3" t="n">
-        <v>170</v>
+        <v>40</v>
       </c>
       <c r="J3" t="n">
-        <v>144</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
@@ -594,27 +594,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0,930</t>
+          <t>0,879</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0,942</t>
+          <t>0,892</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0,936</t>
+          <t>0,885</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0,997</t>
+          <t>0,984</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2595,000</t>
+          <t>398,000</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -623,13 +623,13 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2445</v>
+        <v>355</v>
       </c>
       <c r="I4" t="n">
-        <v>185</v>
+        <v>49</v>
       </c>
       <c r="J4" t="n">
-        <v>150</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -640,42 +640,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0,929</t>
+          <t>0,902</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0,936</t>
+          <t>0,897</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0,933</t>
+          <t>0,899</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0,998</t>
+          <t>0,999</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2555,000</t>
+          <t>399,000</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0,54</t>
+          <t>0,55</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>2391</v>
+        <v>358</v>
       </c>
       <c r="I5" t="n">
-        <v>182</v>
+        <v>39</v>
       </c>
       <c r="J5" t="n">
-        <v>164</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6">
@@ -686,42 +686,42 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0,606</t>
+          <t>0,592</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0,604</t>
+          <t>0,589</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0,605</t>
+          <t>0,591</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>0,999</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2575,000</t>
+          <t>404,000</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0,55</t>
+          <t>0,56</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1555</v>
+        <v>238</v>
       </c>
       <c r="I6" t="n">
-        <v>1011</v>
+        <v>164</v>
       </c>
       <c r="J6" t="n">
-        <v>1020</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7">
@@ -732,17 +732,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0,585</t>
+          <t>0,571</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0,584</t>
+          <t>0,586</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0,585</t>
+          <t>0,579</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -752,135 +752,135 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2518,000</t>
+          <t>377,000</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>0,54</t>
+          <t>0,52</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1471</v>
+        <v>221</v>
       </c>
       <c r="I7" t="n">
-        <v>1044</v>
+        <v>166</v>
       </c>
       <c r="J7" t="n">
-        <v>1047</v>
+        <v>156</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ligature method</t>
+          <t>oral hygiene</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0,703</t>
+          <t>0,865</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0,726</t>
+          <t>0,894</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0,714</t>
+          <t>0,879</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0,998</t>
+          <t>0,978</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1558,000</t>
+          <t>265,000</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0,33</t>
+          <t>0,37</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>1131</v>
+        <v>237</v>
       </c>
       <c r="I8" t="n">
-        <v>478</v>
+        <v>37</v>
       </c>
       <c r="J8" t="n">
-        <v>427</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>oral hygiene</t>
+          <t>ligature method</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0,870</t>
+          <t>0,602</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0,935</t>
+          <t>0,592</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0,901</t>
+          <t>0,597</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>0,995</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1704,000</t>
+          <t>289,000</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0,36</t>
+          <t>0,40</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>1594</v>
+        <v>171</v>
       </c>
       <c r="I9" t="n">
-        <v>239</v>
+        <v>113</v>
       </c>
       <c r="J9" t="n">
-        <v>110</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>elastic pattern left</t>
+          <t>right molar class</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0,818</t>
+          <t>0,870</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0,855</t>
+          <t>0,908</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0,836</t>
+          <t>0,888</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -890,68 +890,68 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1306,000</t>
+          <t>228,000</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0,28</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1116</v>
+        <v>207</v>
       </c>
       <c r="I10" t="n">
-        <v>248</v>
+        <v>31</v>
       </c>
       <c r="J10" t="n">
-        <v>190</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>right canine class</t>
+          <t>left molar class</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0,841</t>
+          <t>0,858</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0,912</t>
+          <t>0,866</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0,875</t>
+          <t>0,862</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0,999</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>1347,000</t>
+          <t>231,000</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>0,29</t>
+          <t>0,32</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1228</v>
+        <v>200</v>
       </c>
       <c r="I11" t="n">
-        <v>232</v>
+        <v>33</v>
       </c>
       <c r="J11" t="n">
-        <v>119</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
@@ -962,17 +962,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0,857</t>
+          <t>0,842</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0,910</t>
+          <t>0,865</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0,883</t>
+          <t>0,853</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -982,1005 +982,963 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1350,000</t>
+          <t>222,000</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>0,29</t>
+          <t>0,31</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1229</v>
+        <v>192</v>
       </c>
       <c r="I12" t="n">
-        <v>205</v>
+        <v>36</v>
       </c>
       <c r="J12" t="n">
-        <v>121</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>right molar class</t>
+          <t>right canine class</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0,872</t>
+          <t>0,851</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0,924</t>
+          <t>0,885</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0,897</t>
+          <t>0,868</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0,999</t>
+          <t>0,998</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1402,000</t>
+          <t>226,000</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>0,30</t>
+          <t>0,31</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1295</v>
+        <v>200</v>
       </c>
       <c r="I13" t="n">
-        <v>190</v>
+        <v>35</v>
       </c>
       <c r="J13" t="n">
-        <v>107</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>left molar class</t>
+          <t>elastic pattern left</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0,879</t>
+          <t>0,702</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>0,922</t>
+          <t>0,780</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0,900</t>
+          <t>0,739</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>0,980</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>1392,000</t>
+          <t>223,000</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0,30</t>
+          <t>0,31</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1284</v>
+        <v>174</v>
       </c>
       <c r="I14" t="n">
-        <v>177</v>
+        <v>74</v>
       </c>
       <c r="J14" t="n">
-        <v>108</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Class II elastic</t>
+          <t>elastic pattern right</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,736</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,799</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,766</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,967</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>234,000</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,33</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>187</v>
+      </c>
+      <c r="I15" t="n">
+        <v>67</v>
+      </c>
+      <c r="J15" t="n">
+        <v>47</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>elastic pattern right</t>
+          <t>compliance</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0,812</t>
+          <t>0,819</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0,854</t>
+          <t>0,839</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0,832</t>
+          <t>0,829</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0,986</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1287,000</t>
+          <t>211,000</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0,27</t>
+          <t>0,29</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1099</v>
+        <v>177</v>
       </c>
       <c r="I16" t="n">
-        <v>255</v>
+        <v>39</v>
       </c>
       <c r="J16" t="n">
-        <v>188</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>compliance</t>
+          <t>elastic type left</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0,842</t>
+          <t>0,886</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0,923</t>
+          <t>0,855</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0,880</t>
+          <t>0,870</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>0,981</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1241,000</t>
+          <t>172,000</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>0,26</t>
+          <t>0,24</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1145</v>
+        <v>147</v>
       </c>
       <c r="I17" t="n">
-        <v>215</v>
+        <v>19</v>
       </c>
       <c r="J17" t="n">
-        <v>96</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>overjet (mm)</t>
+          <t>elastic type right</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0,520</t>
+          <t>0,924</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0,533</t>
+          <t>0,878</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0,527</t>
+          <t>0,901</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0,969</t>
+          <t>0,988</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>910,000</t>
+          <t>181,000</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0,19</t>
+          <t>0,25</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>485</v>
+        <v>159</v>
       </c>
       <c r="I18" t="n">
-        <v>447</v>
+        <v>13</v>
       </c>
       <c r="J18" t="n">
-        <v>425</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>elastic type left</t>
+          <t>overjet (mm)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
+          <t>0,218</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>0,206</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0,212</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>0,899</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>0,913</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>0,906</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>0,988</t>
-        </is>
-      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>951,000</t>
+          <t>165,000</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>0,20</t>
+          <t>0,23</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>868</v>
+        <v>34</v>
       </c>
       <c r="I19" t="n">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="J19" t="n">
-        <v>83</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>elastic type right</t>
+          <t>overbite (mm)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0,889</t>
+          <t>0,203</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0,911</t>
+          <t>0,201</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0,900</t>
+          <t>0,202</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0,989</t>
+          <t>0,862</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>944,000</t>
+          <t>149,000</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0,20</t>
+          <t>0,21</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>860</v>
+        <v>30</v>
       </c>
       <c r="I20" t="n">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="J20" t="n">
-        <v>84</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>overbite (mm)</t>
+          <t>recods taken (x-rays; ios; photos, facial scanning)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>0,510</t>
+          <t>0,652</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0,526</t>
+          <t>0,819</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0,518</t>
+          <t>0,726</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0,960</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>848,000</t>
+          <t>105,000</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0,18</t>
+          <t>0,15</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>446</v>
+        <v>86</v>
       </c>
       <c r="I21" t="n">
-        <v>429</v>
+        <v>46</v>
       </c>
       <c r="J21" t="n">
-        <v>402</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>debonded bracket</t>
+          <t>upper arch bends</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0,733</t>
+          <t>0,641</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0,845</t>
+          <t>0,710</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0,785</t>
+          <t>0,673</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0,998</t>
+          <t>0,956</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>445,000</t>
+          <t>93,000</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>0,09</t>
+          <t>0,13</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>376</v>
+        <v>66</v>
       </c>
       <c r="I22" t="n">
-        <v>137</v>
+        <v>37</v>
       </c>
       <c r="J22" t="n">
-        <v>69</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Lower Retainer</t>
+          <t>lower arch bends</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,634</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,732</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,680</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>71,000</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,10</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>52</v>
+      </c>
+      <c r="I23" t="n">
+        <v>30</v>
+      </c>
+      <c r="J23" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>emergency type</t>
+          <t>debonded bracket</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0,722</t>
+          <t>0,676</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0,573</t>
+          <t>0,738</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0,639</t>
+          <t>0,706</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0,994</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>321,000</t>
+          <t>65,000</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0,07</t>
+          <t>0,09</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>184</v>
+        <v>48</v>
       </c>
       <c r="I24" t="n">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="J24" t="n">
-        <v>137</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Upper Retainer</t>
+          <t>retainer check</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,825</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,855</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,839</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,08</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>47</v>
+      </c>
+      <c r="I25" t="n">
+        <v>10</v>
+      </c>
+      <c r="J25" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Space closure sliding mechanics</t>
+          <t>re-tie appointment</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,643</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,202</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,308</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>89,000</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,12</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>18</v>
+      </c>
+      <c r="I26" t="n">
+        <v>10</v>
+      </c>
+      <c r="J26" t="n">
+        <v>71</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Photos taken</t>
+          <t>appliance</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,536</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,652</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,588</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,855</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>46,000</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,06</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>30</v>
+      </c>
+      <c r="I27" t="n">
+        <v>26</v>
+      </c>
+      <c r="J27" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>upper arch bends</t>
+          <t>emergency type</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0,748</t>
+          <t>0,625</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>0,865</t>
+          <t>0,490</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0,802</t>
+          <t>0,549</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0,988</t>
+          <t>0,941</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>539,000</t>
+          <t>51,000</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>0,11</t>
+          <t>0,07</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>466</v>
+        <v>25</v>
       </c>
       <c r="I28" t="n">
-        <v>157</v>
+        <v>15</v>
       </c>
       <c r="J28" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Class I elastic</t>
+          <t>prescription and bracket slot</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,700</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,420</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,525</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,924</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>50,000</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,07</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>21</v>
+      </c>
+      <c r="I29" t="n">
+        <v>9</v>
+      </c>
+      <c r="J29" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Class III elastic</t>
+          <t>bracket or band repositioning</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,725</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,690</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,707</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,984</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>42,000</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,06</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>29</v>
+      </c>
+      <c r="I30" t="n">
+        <v>11</v>
+      </c>
+      <c r="J30" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>appliance</t>
+          <t>retainer</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0,732</t>
+          <t>0,312</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>0,764</t>
+          <t>0,441</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0,747</t>
+          <t>0,366</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>0,982</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>339,000</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>0,07</t>
+          <t>0,05</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>259</v>
+        <v>15</v>
       </c>
       <c r="I31" t="n">
-        <v>95</v>
+        <v>33</v>
       </c>
       <c r="J31" t="n">
-        <v>80</v>
+        <v>19</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>lower arch bends</t>
+          <t>cos lower</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0,754</t>
+          <t>0,610</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0,863</t>
+          <t>0,735</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0,805</t>
+          <t>0,667</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>0,960</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>459,000</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0,10</t>
+          <t>0,05</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>396</v>
+        <v>25</v>
       </c>
       <c r="I32" t="n">
-        <v>129</v>
+        <v>16</v>
       </c>
       <c r="J32" t="n">
-        <v>63</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>retainer check</t>
+          <t>emergency</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0,910</t>
+          <t>0,824</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0,875</t>
+          <t>0,700</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0,892</t>
+          <t>0,757</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1990,157 +1948,145 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>369,000</t>
+          <t>40,000</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>0,08</t>
+          <t>0,06</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>323</v>
+        <v>28</v>
       </c>
       <c r="I33" t="n">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="J33" t="n">
-        <v>46</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Xrays taken</t>
+          <t>upper bonding</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,684</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,788</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,732</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,978</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>33,000</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,05</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>26</v>
+      </c>
+      <c r="I34" t="n">
+        <v>12</v>
+      </c>
+      <c r="J34" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Intra Oral Scanning Taken</t>
+          <t>ipr</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,838</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,939</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,886</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>33,000</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,05</t>
+        </is>
+      </c>
+      <c r="H35" t="n">
+        <v>31</v>
+      </c>
+      <c r="I35" t="n">
+        <v>6</v>
+      </c>
+      <c r="J35" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>emergency</t>
+          <t>lower bonding</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0,868</t>
+          <t>0,821</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0,771</t>
+          <t>0,639</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0,817</t>
+          <t>0,719</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>0,976</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>231,000</t>
+          <t>36,000</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2149,188 +2095,182 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>178</v>
+        <v>23</v>
       </c>
       <c r="I36" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="J36" t="n">
-        <v>53</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Lower Arch Reverse Curve of Spee</t>
+          <t>open spring</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,750</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,818</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,783</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22,000</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,03</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>18</v>
+      </c>
+      <c r="I37" t="n">
+        <v>6</v>
+      </c>
+      <c r="J37" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>bracket or band repositioning</t>
+          <t>active space closure</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0,793</t>
+          <t>0,529</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0,734</t>
+          <t>0,209</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>0,762</t>
+          <t>0,300</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>0,998</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>308,000</t>
+          <t>43,000</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>0,07</t>
+          <t>0,06</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>226</v>
+        <v>9</v>
       </c>
       <c r="I38" t="n">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="J38" t="n">
-        <v>82</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>open spring</t>
+          <t>cos upper</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>0,831</t>
+          <t>0,625</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0,888</t>
+          <t>0,588</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>0,858</t>
+          <t>0,606</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>0,878</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>205,000</t>
+          <t>17,000</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,02</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>182</v>
+        <v>10</v>
       </c>
       <c r="I39" t="n">
-        <v>37</v>
+        <v>6</v>
       </c>
       <c r="J39" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>upper bonding</t>
+          <t>posterior bite turbos</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>0,780</t>
+          <t>0,514</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0,829</t>
+          <t>0,731</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0,804</t>
+          <t>0,603</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>0,996</t>
+          <t>0,955</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>210,000</t>
+          <t>26,000</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2339,80 +2279,80 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>174</v>
+        <v>19</v>
       </c>
       <c r="I40" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="J40" t="n">
-        <v>36</v>
+        <v>7</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ipr</t>
+          <t>upper debond</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>0,831</t>
+          <t>0,840</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0,933</t>
+          <t>0,875</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>0,879</t>
+          <t>0,857</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>0,998</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>210,000</t>
+          <t>24,000</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>196</v>
+        <v>21</v>
       </c>
       <c r="I41" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="J41" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>re-tie appointment</t>
+          <t>lower debond</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>0,798</t>
+          <t>0,840</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0,371</t>
+          <t>0,955</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>0,507</t>
+          <t>0,894</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2422,239 +2362,227 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>350,000</t>
+          <t>22,000</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>0,07</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>130</v>
+        <v>21</v>
       </c>
       <c r="I42" t="n">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="J42" t="n">
-        <v>220</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>lower bonding</t>
+          <t>enameloplasty</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>0,820</t>
+          <t>0,947</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0,761</t>
+          <t>0,783</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>0,789</t>
+          <t>0,857</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>0,996</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>209,000</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>0,04</t>
+          <t>0,03</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>159</v>
+        <v>18</v>
       </c>
       <c r="I43" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="J43" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>posterior bite turbos</t>
+          <t>tads</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>0,733</t>
+          <t>0,192</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0,859</t>
+          <t>0,556</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0,791</t>
+          <t>0,286</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>0,945</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>163,000</t>
+          <t>9,000</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,01</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>140</v>
+        <v>5</v>
       </c>
       <c r="I44" t="n">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="J44" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Cross Elastic</t>
+          <t>relapse</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,667</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,421</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,516</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,964</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,03</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>8</v>
+      </c>
+      <c r="I45" t="n">
+        <v>4</v>
+      </c>
+      <c r="J45" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Upper Arch Accentuated Curve of Spee</t>
+          <t>tmj symptoms</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,429</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,429</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,429</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,963</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,000</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,02</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>6</v>
+      </c>
+      <c r="I46" t="n">
+        <v>8</v>
+      </c>
+      <c r="J46" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>upper debond</t>
+          <t>upper banding</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>0,914</t>
+          <t>0,727</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0,914</t>
+          <t>0,500</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>0,914</t>
+          <t>0,593</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2664,181 +2592,181 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>140,000</t>
+          <t>16,000</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,02</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="I47" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="J47" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>lower debond</t>
+          <t>tpa</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>0,930</t>
+          <t>0,692</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0,957</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>0,943</t>
+          <t>0,818</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>0,692</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>138,000</t>
+          <t>9,000</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,01</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>132</v>
+        <v>9</v>
       </c>
       <c r="I48" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J48" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>tads</t>
+          <t>referral</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>0,611</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0,727</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>0,664</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0,997</t>
+          <t>0,917</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>110,000</t>
+          <t>3,000</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>0,02</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="H49" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="I49" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="J49" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>prescription and bracket slot</t>
+          <t>extractions</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>0,809</t>
+          <t>0,250</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0,660</t>
+          <t>0,100</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>0,727</t>
+          <t>0,143</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0,990</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>315,000</t>
+          <t>10,000</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>0,07</t>
+          <t>0,01</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>208</v>
+        <v>1</v>
       </c>
       <c r="I50" t="n">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="J50" t="n">
-        <v>107</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>tmj symptoms</t>
+          <t>posterior crossbite</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>0,581</t>
+          <t>0,571</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0,549</t>
+          <t>0,444</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>0,565</t>
+          <t>0,500</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2848,43 +2776,43 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>91,000</t>
+          <t>9,000</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>0,02</t>
+          <t>0,01</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="I51" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="J51" t="n">
-        <v>41</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>enameloplasty</t>
+          <t>lower banding</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>0,860</t>
+          <t>0,750</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0,780</t>
+          <t>0,500</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0,818</t>
+          <t>0,600</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2894,187 +2822,181 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>118,000</t>
+          <t>6,000</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>0,03</t>
+          <t>0,01</t>
         </is>
       </c>
       <c r="H52" t="n">
-        <v>92</v>
+        <v>3</v>
       </c>
       <c r="I52" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="J52" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>referral</t>
+          <t>closed spring</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>0,537</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0,361</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0,431</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>0,956</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>61,000</t>
+          <t>1,000</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>0,01</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="H53" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="J53" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Unilateral Posterior Crossbite</t>
+          <t>anterior bite turbos</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>0,00</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" t="n">
+        <v>2</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>extractions</t>
+          <t>maxillary expander</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>0,667</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0,542</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>0,598</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>0,918</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>0,01</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="I55" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="J55" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>tpa</t>
+          <t>anterior crossbite</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>0,704</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>0,803</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>0,750</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3084,28 +3006,28 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>71,000</t>
+          <t>6,000</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>0,02</t>
+          <t>0,01</t>
         </is>
       </c>
       <c r="H56" t="n">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="I56" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="J56" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Space closure loop mechanics</t>
+          <t>LLHA</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3157,99 +3079,105 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>upper banding</t>
+          <t>mandibular advancement appliance</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>0,714</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>0,526</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>0,606</t>
+          <t>0,000</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>0,991</t>
+          <t>0,794</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>76,000</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>0,02</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="H58" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="J58" t="n">
-        <v>36</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>relapse</t>
+          <t>NANCE</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>0,571</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0,454</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>0,506</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>97,000</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>0,02</t>
-        </is>
-      </c>
-      <c r="H59" t="n">
-        <v>44</v>
-      </c>
-      <c r="I59" t="n">
-        <v>33</v>
-      </c>
-      <c r="J59" t="n">
-        <v>53</v>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Upper Active movement</t>
+          <t>Cantilever</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3301,7 +3229,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Lower Active movement</t>
+          <t>Tongue Crib</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3353,996 +3281,50 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>closed spring</t>
+          <t>FaceMask</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>0,617</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>0,860</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>0,718</t>
+          <t>-</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>1,000</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>43,000</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>0,01</t>
-        </is>
-      </c>
-      <c r="H62" t="n">
-        <v>37</v>
-      </c>
-      <c r="I62" t="n">
-        <v>23</v>
-      </c>
-      <c r="J62" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>lower banding</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>0,806</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>0,556</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>0,658</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>0,984</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>45,000</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>0,01</t>
-        </is>
-      </c>
-      <c r="H63" t="n">
-        <v>25</v>
-      </c>
-      <c r="I63" t="n">
-        <v>6</v>
-      </c>
-      <c r="J63" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Patient ID.1</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>NiTi Closing Spring</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>anterior bite turbos</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>0,857</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>0,500</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>0,632</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>0,911</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>36,000</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>0,01</t>
-        </is>
-      </c>
-      <c r="H66" t="n">
-        <v>18</v>
-      </c>
-      <c r="I66" t="n">
-        <v>3</v>
-      </c>
-      <c r="J66" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>TADs.1</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Upper Arch Reverse Curve of Spee</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>maxillary expander</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>0,477</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>0,677</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>0,560</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>0,982</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>31,000</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>0,01</t>
-        </is>
-      </c>
-      <c r="H69" t="n">
-        <v>21</v>
-      </c>
-      <c r="I69" t="n">
-        <v>23</v>
-      </c>
-      <c r="J69" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>llha</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>1,000</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>0,917</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>0,957</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>0,917</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="H70" t="n">
-        <v>11</v>
-      </c>
-      <c r="I70" t="n">
-        <v>0</v>
-      </c>
-      <c r="J70" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>anterior crossbite</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>0,667</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>0,308</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>0,421</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>1,000</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>13,000</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="H71" t="n">
-        <v>4</v>
-      </c>
-      <c r="I71" t="n">
-        <v>2</v>
-      </c>
-      <c r="J71" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Debonded Bracket/Band</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Lower Arch Curve of Spee</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Intrusion Arch</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Bilateral Posterior Crossbite</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Lower Arch Accentuated Curve of Spee</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Active Traction</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Active Tooth Traction</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>mandibular advancement appliance</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>0,182</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>0,200</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>0,190</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>0,974</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>10,000</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="H79" t="n">
-        <v>2</v>
-      </c>
-      <c r="I79" t="n">
-        <v>9</v>
-      </c>
-      <c r="J79" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Teeth Pain</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Arch Coordination</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4404,22 +3386,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0,746</t>
+          <t>0,598</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0,991</t>
+          <t>0,950</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0,815</t>
+          <t>0,745</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0,995</t>
+          <t>0,984</t>
         </is>
       </c>
     </row>
@@ -4482,7 +3464,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4698</v>
+        <v>720</v>
       </c>
     </row>
     <row r="5">
@@ -4492,7 +3474,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -4502,7 +3484,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>80</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>